<commit_message>
feat(timing_char/work): add wire-delay-per-mm rows to characterization sheet
Adds a new section to the characterization sheet for cross-partition route
budgeting. ASAP7 NLDM has no wire_load table - ABC measures gate delay only -
so these are 7nm industry rules-of-thumb for *buffered* routes:

  M2/M3 (local/intermediate)  120 ps/mm TT
  M4/M5 (semi-global)          65 ps/mm TT
  M6/M7 (global)               40 ps/mm TT
  M8/M9 (thick)                22 ps/mm TT

Corner scaling applied via TT/FF/SS columns: FF = 0.80x TT, SS = 1.30x TT
(resistance rises with temperature).  Numbers are distance-based and so are
freq-independent; repeated across the freq columns for sheet uniformity.

When a FUB output crosses a partition boundary, look up the destination
metal layer here and add (route_length_mm * ps_per_mm) to the data->D
delay column on the building-blocks / stream sheets.
</commit_message>
<xml_diff>
--- a/projects/components/timing_characterization/work/asap7_characterization.xlsx
+++ b/projects/components/timing_characterization/work/asap7_characterization.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1248,56 +1248,227 @@
       <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Wire delay per mm by metal layer (buffered route, ps/mm) - cross-partition route estimate</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Probe corner_freq columns are independent measurements (see Per-level table above).</t>
-        </is>
+          <t>M2/M3 (local / intermediate)</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>120</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="G28" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>156</v>
+      </c>
+      <c r="I28" s="2" t="n">
+        <v>156</v>
+      </c>
+      <c r="J28" s="2" t="n">
+        <v>156</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Tflop = Tcq + Tsu derived from NAND chain two-point probe (LEVELS={3,6}).</t>
-        </is>
+          <t>M4/M5 (semi-global)</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="G29" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="I29" s="2" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="J29" s="2" t="n">
+        <v>84.5</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>max_levels = floor((period_ps - Tflop) / per_level_delay).</t>
-        </is>
+          <t>M6/M7 (global)</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="G30" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="I30" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="J30" s="2" t="n">
+        <v>52</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>** When the critical path is a mixed bag of cells (typical for datapath / FSM next-state / arbitration logic), use the MULT per-level number. It bakes in AND / XOR / full-adder / carry mix.</t>
-        </is>
+          <t>M8/M9 (thick)</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="F31" s="2" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="G31" s="2" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="I31" s="2" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="J31" s="2" t="n">
+        <v>28.6</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>INV: ABC's strash collapses inverter pairs across the chain, so lev doesn't change between probe sizes - per-level slope is degenerate. Single-point delay is reported in the reference table.</t>
-        </is>
-      </c>
+      <c r="A32" t="inlineStr"/>
+      <c r="B32" t="inlineStr"/>
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>CLK_DIV: critical path is intra-stage (counter + pickoff), so NUM_STAGES doesn't move lev. Single-point delay is reported in the reference table.</t>
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
+        <is>
+          <t>Probe corner_freq columns are independent measurements (see Per-level table above).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Tflop = Tcq + Tsu derived from NAND chain two-point probe (LEVELS={3,6}).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>max_levels = floor((period_ps - Tflop) / per_level_delay).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>** When the critical path is a mixed bag of cells (typical for datapath / FSM next-state / arbitration logic), use the MULT per-level number. It bakes in AND / XOR / full-adder / carry mix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>INV: ABC's strash collapses inverter pairs across the chain, so lev doesn't change between probe sizes - per-level slope is degenerate. Single-point delay is reported in the reference table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>CLK_DIV: critical path is intra-stage (counter + pickoff), so NUM_STAGES doesn't move lev. Single-point delay is reported in the reference table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Wire delays are 7nm industry rule-of-thumb for buffered routes; the ASAP7 NLDM ships no wire_load table so ABC measured gate delay only. For partition-to-partition output budgeting, look up the destination metal layer and multiply by route length (mm).</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Raw probe data is in work/timing_char_data.csv. Reproducer is work/timing_char_sweep.py.</t>
         </is>

</xml_diff>

<commit_message>
feat(timing_char/work): shift sweep grid to 1.0/1.25/1.5/1.75/2.0 GHz
User wants the methodology to illustrate paths going from passing to
failing.  The old 500/750/1000 MHz sweep keeps everything comfortably
passing for an ASAP7 7nm characterization.  Pushing the grid to where
modern designs hit the wall:

  columns: TT_1000 / TT_1250 / TT_1500 / TT_1750 / TT_2000
           FF_1000 / FF_1250 / FF_1500 / FF_1750 / FF_2000
           SS_1000 / SS_1250 / SS_1500 / SS_1750 / SS_2000

Sample TT-corner Max-levels-per-cycle ranges over the new sweep:
  NAND:  135 ->  66     (47% drop)
  MUX:    60 ->  29
  XOR:    36 ->  18
  MULT:   32 ->  16     (PROXY for mixed-bag logic)
  CARRY:  31 ->  15

Cell refs into the characterization sheet bumped to match the new column
layout: per_NAND TT is now $B$15 (was $D$15 when TT_1000 was col D);
FF stays $G$15 (lucky col coincidence); SS $L$15 (was $J$15). Both
building blocks and stream sheets updated to point at the new columns.
</commit_message>
<xml_diff>
--- a/projects/components/timing_characterization/work/asap7_characterization.xlsx
+++ b/projects/components/timing_characterization/work/asap7_characterization.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J50"/>
+  <dimension ref="A1:P50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -496,6 +496,12 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,27 +512,27 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>TT_500MHz</t>
+          <t>TT_1000MHz</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>TT_750MHz</t>
+          <t>TT_1250MHz</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>TT_1000MHz</t>
+          <t>TT_1500MHz</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>FF_500MHz</t>
+          <t>TT_1750MHz</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>FF_750MHz</t>
+          <t>TT_2000MHz</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -536,17 +542,47 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>SS_500MHz</t>
+          <t>FF_1250MHz</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>SS_750MHz</t>
+          <t>FF_1500MHz</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>FF_1750MHz</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>FF_2000MHz</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>SS_1000MHz</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>SS_1250MHz</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>SS_1500MHz</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>SS_1750MHz</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>SS_2000MHz</t>
         </is>
       </c>
     </row>
@@ -557,31 +593,49 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1333.3</v>
+        <v>800</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1000</v>
+        <v>666.7</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2000</v>
+        <v>571.4</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>1333.3</v>
+        <v>500</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>1000</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>2000</v>
+        <v>800</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>1333.3</v>
+        <v>666.7</v>
       </c>
       <c r="J2" s="2" t="n">
+        <v>571.4</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="L2" s="2" t="n">
         <v>1000</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>800</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>666.7</v>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>571.4</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="3">
@@ -600,21 +654,39 @@
         <v>16.59</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>10.53</v>
+        <v>16.59</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>10.53</v>
+        <v>16.59</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>10.53</v>
       </c>
       <c r="H3" s="2" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>10.53</v>
+      </c>
+      <c r="L3" s="2" t="n">
         <v>22.73</v>
       </c>
-      <c r="I3" s="2" t="n">
+      <c r="M3" s="2" t="n">
         <v>22.73</v>
       </c>
-      <c r="J3" s="2" t="n">
+      <c r="N3" s="2" t="n">
+        <v>22.73</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>22.73</v>
+      </c>
+      <c r="P3" s="2" t="n">
         <v>22.73</v>
       </c>
     </row>
@@ -629,6 +701,12 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -645,6 +723,12 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -653,31 +737,49 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>273</v>
+        <v>135</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>181</v>
+        <v>107</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>135</v>
+        <v>89</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>335</v>
+        <v>76</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>223</v>
+        <v>66</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>166</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>172</v>
+        <v>133</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="J6" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="L6" s="2" t="n">
         <v>85</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="O6" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="P6" s="2" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="7">
@@ -687,19 +789,19 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>74</v>
+        <v>36</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>124</v>
+        <v>20</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>82</v>
+        <v>18</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>61</v>
@@ -708,10 +810,28 @@
         <v>49</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="J7" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="L7" s="2" t="n">
         <v>24</v>
+      </c>
+      <c r="M7" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="O7" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="P7" s="2" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -721,31 +841,49 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>121</v>
+        <v>60</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>80</v>
+        <v>48</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>180</v>
+        <v>34</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>120</v>
+        <v>29</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>89</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="J8" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="L8" s="2" t="n">
         <v>39</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="N8" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="O8" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="P8" s="2" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="9">
@@ -755,31 +893,49 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>64</v>
+        <v>31</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>94</v>
+        <v>18</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>63</v>
+        <v>15</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>47</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="J9" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="L9" s="2" t="n">
         <v>21</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="O9" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="P9" s="2" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="10">
@@ -789,31 +945,49 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>66</v>
+        <v>32</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>91</v>
+        <v>18</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="G10" s="5" t="n">
         <v>45</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="J10" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="L10" s="5" t="n">
         <v>26</v>
+      </c>
+      <c r="M10" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="N10" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="O10" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="P10" s="5" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="11">
@@ -823,31 +997,49 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>14</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="J11" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="L11" s="2" t="n">
         <v>10</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="N11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -857,31 +1049,49 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>171</v>
+        <v>84</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>113</v>
+        <v>67</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>24</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="J12" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L12" s="2" t="n">
         <v>18</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="N12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="O12" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="P12" s="2" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -895,6 +1105,12 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -911,6 +1127,12 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -928,21 +1150,39 @@
         <v>7.25</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>5.93</v>
+        <v>7.25</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>5.93</v>
+        <v>7.25</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>5.93</v>
       </c>
       <c r="H15" s="2" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>5.93</v>
+      </c>
+      <c r="L15" s="2" t="n">
         <v>11.47</v>
       </c>
-      <c r="I15" s="2" t="n">
+      <c r="M15" s="2" t="n">
         <v>11.47</v>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="N15" s="2" t="n">
+        <v>11.47</v>
+      </c>
+      <c r="O15" s="2" t="n">
+        <v>11.47</v>
+      </c>
+      <c r="P15" s="2" t="n">
         <v>11.47</v>
       </c>
     </row>
@@ -962,21 +1202,39 @@
         <v>26.77</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>16.01</v>
+        <v>26.77</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>16.01</v>
+        <v>26.77</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>16.01</v>
       </c>
       <c r="H16" s="2" t="n">
+        <v>16.01</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>16.01</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>16.01</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>16.01</v>
+      </c>
+      <c r="L16" s="2" t="n">
         <v>39.69</v>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="M16" s="2" t="n">
         <v>39.69</v>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="N16" s="2" t="n">
+        <v>39.69</v>
+      </c>
+      <c r="O16" s="2" t="n">
+        <v>39.69</v>
+      </c>
+      <c r="P16" s="2" t="n">
         <v>39.69</v>
       </c>
     </row>
@@ -996,21 +1254,39 @@
         <v>16.29</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>11</v>
+        <v>16.29</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>11</v>
+        <v>16.29</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>11</v>
       </c>
       <c r="H17" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="L17" s="2" t="n">
         <v>24.97</v>
       </c>
-      <c r="I17" s="2" t="n">
+      <c r="M17" s="2" t="n">
         <v>24.97</v>
       </c>
-      <c r="J17" s="2" t="n">
+      <c r="N17" s="2" t="n">
+        <v>24.97</v>
+      </c>
+      <c r="O17" s="2" t="n">
+        <v>24.97</v>
+      </c>
+      <c r="P17" s="2" t="n">
         <v>24.97</v>
       </c>
     </row>
@@ -1030,21 +1306,39 @@
         <v>30.77</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>20.97</v>
+        <v>30.77</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>20.97</v>
+        <v>30.77</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>20.97</v>
       </c>
       <c r="H18" s="2" t="n">
+        <v>20.97</v>
+      </c>
+      <c r="I18" s="2" t="n">
+        <v>20.97</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>20.97</v>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>20.97</v>
+      </c>
+      <c r="L18" s="2" t="n">
         <v>45.22</v>
       </c>
-      <c r="I18" s="2" t="n">
+      <c r="M18" s="2" t="n">
         <v>45.22</v>
       </c>
-      <c r="J18" s="2" t="n">
+      <c r="N18" s="2" t="n">
+        <v>45.22</v>
+      </c>
+      <c r="O18" s="2" t="n">
+        <v>45.22</v>
+      </c>
+      <c r="P18" s="2" t="n">
         <v>45.22</v>
       </c>
     </row>
@@ -1064,21 +1358,39 @@
         <v>29.95</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>21.75</v>
+        <v>29.95</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>21.75</v>
+        <v>29.95</v>
       </c>
       <c r="G19" s="5" t="n">
         <v>21.75</v>
       </c>
       <c r="H19" s="5" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>21.75</v>
+      </c>
+      <c r="L19" s="5" t="n">
         <v>37.44</v>
       </c>
-      <c r="I19" s="5" t="n">
+      <c r="M19" s="5" t="n">
         <v>37.44</v>
       </c>
-      <c r="J19" s="5" t="n">
+      <c r="N19" s="5" t="n">
+        <v>37.44</v>
+      </c>
+      <c r="O19" s="5" t="n">
+        <v>37.44</v>
+      </c>
+      <c r="P19" s="5" t="n">
         <v>37.44</v>
       </c>
     </row>
@@ -1098,21 +1410,39 @@
         <v>58.44</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>66.65000000000001</v>
+        <v>58.44</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>66.65000000000001</v>
+        <v>58.44</v>
       </c>
       <c r="G20" s="2" t="n">
         <v>66.65000000000001</v>
       </c>
       <c r="H20" s="2" t="n">
+        <v>66.65000000000001</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>66.65000000000001</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>66.65000000000001</v>
+      </c>
+      <c r="K20" s="2" t="n">
+        <v>66.65000000000001</v>
+      </c>
+      <c r="L20" s="2" t="n">
         <v>90.34</v>
       </c>
-      <c r="I20" s="2" t="n">
+      <c r="M20" s="2" t="n">
         <v>90.34</v>
       </c>
-      <c r="J20" s="2" t="n">
+      <c r="N20" s="2" t="n">
+        <v>90.34</v>
+      </c>
+      <c r="O20" s="2" t="n">
+        <v>90.34</v>
+      </c>
+      <c r="P20" s="2" t="n">
         <v>90.34</v>
       </c>
     </row>
@@ -1132,21 +1462,39 @@
         <v>11.57</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>40.17</v>
+        <v>11.57</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>40.17</v>
+        <v>11.57</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>40.17</v>
       </c>
       <c r="H21" s="2" t="n">
+        <v>40.17</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>40.17</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>40.17</v>
+      </c>
+      <c r="K21" s="2" t="n">
+        <v>40.17</v>
+      </c>
+      <c r="L21" s="2" t="n">
         <v>54.23</v>
       </c>
-      <c r="I21" s="2" t="n">
+      <c r="M21" s="2" t="n">
         <v>54.23</v>
       </c>
-      <c r="J21" s="2" t="n">
+      <c r="N21" s="2" t="n">
+        <v>54.23</v>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>54.23</v>
+      </c>
+      <c r="P21" s="2" t="n">
         <v>54.23</v>
       </c>
     </row>
@@ -1161,6 +1509,12 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1177,6 +1531,12 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1194,21 +1554,39 @@
         <v>14.47</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>12.22</v>
+        <v>14.47</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>12.22</v>
+        <v>14.47</v>
       </c>
       <c r="G24" s="2" t="n">
         <v>12.22</v>
       </c>
       <c r="H24" s="2" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="I24" s="2" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="J24" s="2" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="K24" s="2" t="n">
+        <v>12.22</v>
+      </c>
+      <c r="L24" s="2" t="n">
         <v>22.33</v>
       </c>
-      <c r="I24" s="2" t="n">
+      <c r="M24" s="2" t="n">
         <v>22.33</v>
       </c>
-      <c r="J24" s="2" t="n">
+      <c r="N24" s="2" t="n">
+        <v>22.33</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>22.33</v>
+      </c>
+      <c r="P24" s="2" t="n">
         <v>22.33</v>
       </c>
     </row>
@@ -1228,21 +1606,39 @@
         <v>21.05</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>16.61</v>
+        <v>21.05</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>16.61</v>
+        <v>21.05</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>16.61</v>
       </c>
       <c r="H25" s="2" t="n">
+        <v>16.61</v>
+      </c>
+      <c r="I25" s="2" t="n">
+        <v>16.61</v>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>16.61</v>
+      </c>
+      <c r="K25" s="2" t="n">
+        <v>16.61</v>
+      </c>
+      <c r="L25" s="2" t="n">
         <v>31.29</v>
       </c>
-      <c r="I25" s="2" t="n">
+      <c r="M25" s="2" t="n">
         <v>31.29</v>
       </c>
-      <c r="J25" s="2" t="n">
+      <c r="N25" s="2" t="n">
+        <v>31.29</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>31.29</v>
+      </c>
+      <c r="P25" s="2" t="n">
         <v>31.29</v>
       </c>
     </row>
@@ -1257,6 +1653,12 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1273,6 +1675,12 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -1429,6 +1837,12 @@
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -1445,6 +1859,12 @@
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1462,21 +1882,39 @@
         <v>120</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>96</v>
       </c>
       <c r="H37" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="I37" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="J37" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="K37" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="L37" s="2" t="n">
         <v>156</v>
       </c>
-      <c r="I37" s="2" t="n">
+      <c r="M37" s="2" t="n">
         <v>156</v>
       </c>
-      <c r="J37" s="2" t="n">
+      <c r="N37" s="2" t="n">
+        <v>156</v>
+      </c>
+      <c r="O37" s="2" t="n">
+        <v>156</v>
+      </c>
+      <c r="P37" s="2" t="n">
         <v>156</v>
       </c>
     </row>
@@ -1496,21 +1934,39 @@
         <v>65</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>52</v>
       </c>
       <c r="H38" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="J38" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="K38" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="L38" s="2" t="n">
         <v>84.5</v>
       </c>
-      <c r="I38" s="2" t="n">
+      <c r="M38" s="2" t="n">
         <v>84.5</v>
       </c>
-      <c r="J38" s="2" t="n">
+      <c r="N38" s="2" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="O38" s="2" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="P38" s="2" t="n">
         <v>84.5</v>
       </c>
     </row>
@@ -1530,21 +1986,39 @@
         <v>40</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>32</v>
       </c>
       <c r="H39" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="I39" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="J39" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="K39" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="L39" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="I39" s="2" t="n">
+      <c r="M39" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="J39" s="2" t="n">
+      <c r="N39" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="P39" s="2" t="n">
         <v>52</v>
       </c>
     </row>
@@ -1564,21 +2038,39 @@
         <v>22</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>17.6</v>
+        <v>22</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>17.6</v>
+        <v>22</v>
       </c>
       <c r="G40" s="2" t="n">
         <v>17.6</v>
       </c>
       <c r="H40" s="2" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="I40" s="2" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="J40" s="2" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="K40" s="2" t="n">
+        <v>17.6</v>
+      </c>
+      <c r="L40" s="2" t="n">
         <v>28.6</v>
       </c>
-      <c r="I40" s="2" t="n">
+      <c r="M40" s="2" t="n">
         <v>28.6</v>
       </c>
-      <c r="J40" s="2" t="n">
+      <c r="N40" s="2" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="O40" s="2" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="P40" s="2" t="n">
         <v>28.6</v>
       </c>
     </row>
@@ -1593,6 +2085,12 @@
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
@@ -1919,7 +2417,7 @@
         <v>1</v>
       </c>
       <c r="M4" s="7">
-        <f>K4*characterization!$D$17 + L4*characterization!$D$15</f>
+        <f>K4*characterization!$B$17 + L4*characterization!$B$15</f>
         <v/>
       </c>
       <c r="N4" s="7">
@@ -1927,7 +2425,7 @@
         <v/>
       </c>
       <c r="O4" s="7">
-        <f>K4*characterization!$J$17 + L4*characterization!$J$15</f>
+        <f>K4*characterization!$L$17 + L4*characterization!$L$15</f>
         <v/>
       </c>
       <c r="P4" t="n">
@@ -1937,7 +2435,7 @@
         <v>1</v>
       </c>
       <c r="R4" s="7">
-        <f>P4*characterization!$D$17 + Q4*characterization!$D$15</f>
+        <f>P4*characterization!$B$17 + Q4*characterization!$B$15</f>
         <v/>
       </c>
       <c r="S4" s="7">
@@ -1945,11 +2443,11 @@
         <v/>
       </c>
       <c r="T4" s="7">
-        <f>P4*characterization!$J$17 + Q4*characterization!$J$15</f>
+        <f>P4*characterization!$L$17 + Q4*characterization!$L$15</f>
         <v/>
       </c>
       <c r="U4" s="7">
-        <f>ROUND(1000000/(MAX(M4,R4) + characterization!$D$3), 0)</f>
+        <f>ROUND(1000000/(MAX(M4,R4) + characterization!$B$3), 0)</f>
         <v/>
       </c>
       <c r="V4" s="7">
@@ -1957,7 +2455,7 @@
         <v/>
       </c>
       <c r="W4" s="7">
-        <f>ROUND(1000000/(MAX(O4,T4) + characterization!$J$3), 0)</f>
+        <f>ROUND(1000000/(MAX(O4,T4) + characterization!$L$3), 0)</f>
         <v/>
       </c>
       <c r="X4" s="5" t="inlineStr">
@@ -2031,7 +2529,7 @@
         <v>1</v>
       </c>
       <c r="M5" s="7">
-        <f>K5*characterization!$D$17 + L5*characterization!$D$15</f>
+        <f>K5*characterization!$B$17 + L5*characterization!$B$15</f>
         <v/>
       </c>
       <c r="N5" s="7">
@@ -2039,7 +2537,7 @@
         <v/>
       </c>
       <c r="O5" s="7">
-        <f>K5*characterization!$J$17 + L5*characterization!$J$15</f>
+        <f>K5*characterization!$L$17 + L5*characterization!$L$15</f>
         <v/>
       </c>
       <c r="P5" t="n">
@@ -2049,7 +2547,7 @@
         <v>1</v>
       </c>
       <c r="R5" s="7">
-        <f>P5*characterization!$D$17 + Q5*characterization!$D$15</f>
+        <f>P5*characterization!$B$17 + Q5*characterization!$B$15</f>
         <v/>
       </c>
       <c r="S5" s="7">
@@ -2057,11 +2555,11 @@
         <v/>
       </c>
       <c r="T5" s="7">
-        <f>P5*characterization!$J$17 + Q5*characterization!$J$15</f>
+        <f>P5*characterization!$L$17 + Q5*characterization!$L$15</f>
         <v/>
       </c>
       <c r="U5" s="7">
-        <f>ROUND(1000000/(MAX(M5,R5) + characterization!$D$3), 0)</f>
+        <f>ROUND(1000000/(MAX(M5,R5) + characterization!$B$3), 0)</f>
         <v/>
       </c>
       <c r="V5" s="7">
@@ -2069,7 +2567,7 @@
         <v/>
       </c>
       <c r="W5" s="7">
-        <f>ROUND(1000000/(MAX(O5,T5) + characterization!$J$3), 0)</f>
+        <f>ROUND(1000000/(MAX(O5,T5) + characterization!$L$3), 0)</f>
         <v/>
       </c>
       <c r="X5" s="5" t="inlineStr">
@@ -2150,7 +2648,7 @@
         <v>1</v>
       </c>
       <c r="M7" s="7">
-        <f>K7*characterization!$D$17 + L7*characterization!$D$15</f>
+        <f>K7*characterization!$B$17 + L7*characterization!$B$15</f>
         <v/>
       </c>
       <c r="N7" s="7">
@@ -2158,7 +2656,7 @@
         <v/>
       </c>
       <c r="O7" s="7">
-        <f>K7*characterization!$J$17 + L7*characterization!$J$15</f>
+        <f>K7*characterization!$L$17 + L7*characterization!$L$15</f>
         <v/>
       </c>
       <c r="P7" t="n">
@@ -2168,7 +2666,7 @@
         <v>0</v>
       </c>
       <c r="R7" s="7">
-        <f>P7*characterization!$D$17 + Q7*characterization!$D$15</f>
+        <f>P7*characterization!$B$17 + Q7*characterization!$B$15</f>
         <v/>
       </c>
       <c r="S7" s="7">
@@ -2176,11 +2674,11 @@
         <v/>
       </c>
       <c r="T7" s="7">
-        <f>P7*characterization!$J$17 + Q7*characterization!$J$15</f>
+        <f>P7*characterization!$L$17 + Q7*characterization!$L$15</f>
         <v/>
       </c>
       <c r="U7" s="7">
-        <f>ROUND(1000000/(MAX(M7,R7) + characterization!$D$3), 0)</f>
+        <f>ROUND(1000000/(MAX(M7,R7) + characterization!$B$3), 0)</f>
         <v/>
       </c>
       <c r="V7" s="7">
@@ -2188,7 +2686,7 @@
         <v/>
       </c>
       <c r="W7" s="7">
-        <f>ROUND(1000000/(MAX(O7,T7) + characterization!$J$3), 0)</f>
+        <f>ROUND(1000000/(MAX(O7,T7) + characterization!$L$3), 0)</f>
         <v/>
       </c>
       <c r="X7" s="5" t="inlineStr">
@@ -2262,7 +2760,7 @@
         <v>2</v>
       </c>
       <c r="M8" s="7">
-        <f>K8*characterization!$D$17 + L8*characterization!$D$15</f>
+        <f>K8*characterization!$B$17 + L8*characterization!$B$15</f>
         <v/>
       </c>
       <c r="N8" s="7">
@@ -2270,7 +2768,7 @@
         <v/>
       </c>
       <c r="O8" s="7">
-        <f>K8*characterization!$J$17 + L8*characterization!$J$15</f>
+        <f>K8*characterization!$L$17 + L8*characterization!$L$15</f>
         <v/>
       </c>
       <c r="P8">
@@ -2281,7 +2779,7 @@
         <v>0</v>
       </c>
       <c r="R8" s="7">
-        <f>P8*characterization!$D$17 + Q8*characterization!$D$15</f>
+        <f>P8*characterization!$B$17 + Q8*characterization!$B$15</f>
         <v/>
       </c>
       <c r="S8" s="7">
@@ -2289,11 +2787,11 @@
         <v/>
       </c>
       <c r="T8" s="7">
-        <f>P8*characterization!$J$17 + Q8*characterization!$J$15</f>
+        <f>P8*characterization!$L$17 + Q8*characterization!$L$15</f>
         <v/>
       </c>
       <c r="U8" s="7">
-        <f>ROUND(1000000/(MAX(M8,R8) + characterization!$D$3), 0)</f>
+        <f>ROUND(1000000/(MAX(M8,R8) + characterization!$B$3), 0)</f>
         <v/>
       </c>
       <c r="V8" s="7">
@@ -2301,7 +2799,7 @@
         <v/>
       </c>
       <c r="W8" s="7">
-        <f>ROUND(1000000/(MAX(O8,T8) + characterization!$J$3), 0)</f>
+        <f>ROUND(1000000/(MAX(O8,T8) + characterization!$L$3), 0)</f>
         <v/>
       </c>
       <c r="X8" s="5" t="inlineStr">
@@ -2372,7 +2870,7 @@
         <v>1</v>
       </c>
       <c r="M9" s="7">
-        <f>K9*characterization!$D$17 + L9*characterization!$D$15</f>
+        <f>K9*characterization!$B$17 + L9*characterization!$B$15</f>
         <v/>
       </c>
       <c r="N9" s="7">
@@ -2380,7 +2878,7 @@
         <v/>
       </c>
       <c r="O9" s="7">
-        <f>K9*characterization!$J$17 + L9*characterization!$J$15</f>
+        <f>K9*characterization!$L$17 + L9*characterization!$L$15</f>
         <v/>
       </c>
       <c r="P9">
@@ -2391,7 +2889,7 @@
         <v>1</v>
       </c>
       <c r="R9" s="7">
-        <f>P9*characterization!$D$17 + Q9*characterization!$D$15</f>
+        <f>P9*characterization!$B$17 + Q9*characterization!$B$15</f>
         <v/>
       </c>
       <c r="S9" s="7">
@@ -2399,11 +2897,11 @@
         <v/>
       </c>
       <c r="T9" s="7">
-        <f>P9*characterization!$J$17 + Q9*characterization!$J$15</f>
+        <f>P9*characterization!$L$17 + Q9*characterization!$L$15</f>
         <v/>
       </c>
       <c r="U9" s="7">
-        <f>ROUND(1000000/(MAX(M9,R9) + characterization!$D$3), 0)</f>
+        <f>ROUND(1000000/(MAX(M9,R9) + characterization!$B$3), 0)</f>
         <v/>
       </c>
       <c r="V9" s="7">
@@ -2411,7 +2909,7 @@
         <v/>
       </c>
       <c r="W9" s="7">
-        <f>ROUND(1000000/(MAX(O9,T9) + characterization!$J$3), 0)</f>
+        <f>ROUND(1000000/(MAX(O9,T9) + characterization!$L$3), 0)</f>
         <v/>
       </c>
       <c r="X9" s="5" t="inlineStr">
@@ -2497,7 +2995,7 @@
         <v>1</v>
       </c>
       <c r="M10" s="7">
-        <f>K10*characterization!$D$17 + L10*characterization!$D$15</f>
+        <f>K10*characterization!$B$17 + L10*characterization!$B$15</f>
         <v/>
       </c>
       <c r="N10" s="7">
@@ -2505,7 +3003,7 @@
         <v/>
       </c>
       <c r="O10" s="7">
-        <f>K10*characterization!$J$17 + L10*characterization!$J$15</f>
+        <f>K10*characterization!$L$17 + L10*characterization!$L$15</f>
         <v/>
       </c>
       <c r="P10" t="n">
@@ -2515,7 +3013,7 @@
         <v>1</v>
       </c>
       <c r="R10" s="7">
-        <f>P10*characterization!$D$17 + Q10*characterization!$D$15</f>
+        <f>P10*characterization!$B$17 + Q10*characterization!$B$15</f>
         <v/>
       </c>
       <c r="S10" s="7">
@@ -2523,11 +3021,11 @@
         <v/>
       </c>
       <c r="T10" s="7">
-        <f>P10*characterization!$J$17 + Q10*characterization!$J$15</f>
+        <f>P10*characterization!$L$17 + Q10*characterization!$L$15</f>
         <v/>
       </c>
       <c r="U10" s="7">
-        <f>ROUND(1000000/(MAX(M10,R10) + characterization!$D$3), 0)</f>
+        <f>ROUND(1000000/(MAX(M10,R10) + characterization!$B$3), 0)</f>
         <v/>
       </c>
       <c r="V10" s="7">
@@ -2535,7 +3033,7 @@
         <v/>
       </c>
       <c r="W10" s="7">
-        <f>ROUND(1000000/(MAX(O10,T10) + characterization!$J$3), 0)</f>
+        <f>ROUND(1000000/(MAX(O10,T10) + characterization!$L$3), 0)</f>
         <v/>
       </c>
       <c r="X10" s="5" t="inlineStr">
@@ -2621,7 +3119,7 @@
         <v>1</v>
       </c>
       <c r="M11" s="7">
-        <f>K11*characterization!$D$17 + L11*characterization!$D$15</f>
+        <f>K11*characterization!$B$17 + L11*characterization!$B$15</f>
         <v/>
       </c>
       <c r="N11" s="7">
@@ -2629,7 +3127,7 @@
         <v/>
       </c>
       <c r="O11" s="7">
-        <f>K11*characterization!$J$17 + L11*characterization!$J$15</f>
+        <f>K11*characterization!$L$17 + L11*characterization!$L$15</f>
         <v/>
       </c>
       <c r="P11" t="n">
@@ -2639,7 +3137,7 @@
         <v>1</v>
       </c>
       <c r="R11" s="7">
-        <f>P11*characterization!$D$17 + Q11*characterization!$D$15</f>
+        <f>P11*characterization!$B$17 + Q11*characterization!$B$15</f>
         <v/>
       </c>
       <c r="S11" s="7">
@@ -2647,11 +3145,11 @@
         <v/>
       </c>
       <c r="T11" s="7">
-        <f>P11*characterization!$J$17 + Q11*characterization!$J$15</f>
+        <f>P11*characterization!$L$17 + Q11*characterization!$L$15</f>
         <v/>
       </c>
       <c r="U11" s="7">
-        <f>ROUND(1000000/(MAX(M11,R11) + characterization!$D$3), 0)</f>
+        <f>ROUND(1000000/(MAX(M11,R11) + characterization!$B$3), 0)</f>
         <v/>
       </c>
       <c r="V11" s="7">
@@ -2659,7 +3157,7 @@
         <v/>
       </c>
       <c r="W11" s="7">
-        <f>ROUND(1000000/(MAX(O11,T11) + characterization!$J$3), 0)</f>
+        <f>ROUND(1000000/(MAX(O11,T11) + characterization!$L$3), 0)</f>
         <v/>
       </c>
       <c r="X11" s="5" t="inlineStr">
@@ -2986,7 +3484,7 @@
         </is>
       </c>
       <c r="I4" s="7">
-        <f>F4*characterization!$D$17 + G4*characterization!$D$15</f>
+        <f>F4*characterization!$B$17 + G4*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J4" s="7">
@@ -2994,7 +3492,7 @@
         <v/>
       </c>
       <c r="K4" s="7">
-        <f>F4*characterization!$J$17 + G4*characterization!$J$15</f>
+        <f>F4*characterization!$L$17 + G4*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L4" s="7">
@@ -3065,7 +3563,7 @@
         </is>
       </c>
       <c r="I5" s="7">
-        <f>F5*characterization!$D$17 + G5*characterization!$D$15</f>
+        <f>F5*characterization!$B$17 + G5*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J5" s="7">
@@ -3073,7 +3571,7 @@
         <v/>
       </c>
       <c r="K5" s="7">
-        <f>F5*characterization!$J$17 + G5*characterization!$J$15</f>
+        <f>F5*characterization!$L$17 + G5*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L5" s="7">
@@ -3140,7 +3638,7 @@
         </is>
       </c>
       <c r="I6" s="7">
-        <f>F6*characterization!$D$17 + G6*characterization!$D$15</f>
+        <f>F6*characterization!$B$17 + G6*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J6" s="7">
@@ -3148,7 +3646,7 @@
         <v/>
       </c>
       <c r="K6" s="7">
-        <f>F6*characterization!$J$17 + G6*characterization!$J$15</f>
+        <f>F6*characterization!$L$17 + G6*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L6" s="7">
@@ -3215,7 +3713,7 @@
         </is>
       </c>
       <c r="I7" s="7">
-        <f>F7*characterization!$D$17 + G7*characterization!$D$15</f>
+        <f>F7*characterization!$B$17 + G7*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J7" s="7">
@@ -3223,7 +3721,7 @@
         <v/>
       </c>
       <c r="K7" s="7">
-        <f>F7*characterization!$J$17 + G7*characterization!$J$15</f>
+        <f>F7*characterization!$L$17 + G7*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L7" s="7">
@@ -3294,7 +3792,7 @@
         </is>
       </c>
       <c r="I8" s="7">
-        <f>F8*characterization!$D$17 + G8*characterization!$D$15</f>
+        <f>F8*characterization!$B$17 + G8*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J8" s="7">
@@ -3302,7 +3800,7 @@
         <v/>
       </c>
       <c r="K8" s="7">
-        <f>F8*characterization!$J$17 + G8*characterization!$J$15</f>
+        <f>F8*characterization!$L$17 + G8*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L8" s="7">
@@ -3373,7 +3871,7 @@
         </is>
       </c>
       <c r="I9" s="7">
-        <f>F9*characterization!$D$17 + G9*characterization!$D$15</f>
+        <f>F9*characterization!$B$17 + G9*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J9" s="7">
@@ -3381,7 +3879,7 @@
         <v/>
       </c>
       <c r="K9" s="7">
-        <f>F9*characterization!$J$17 + G9*characterization!$J$15</f>
+        <f>F9*characterization!$L$17 + G9*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L9" s="7">
@@ -3452,7 +3950,7 @@
         </is>
       </c>
       <c r="I10" s="7">
-        <f>F10*characterization!$D$17 + G10*characterization!$D$15</f>
+        <f>F10*characterization!$B$17 + G10*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J10" s="7">
@@ -3460,7 +3958,7 @@
         <v/>
       </c>
       <c r="K10" s="7">
-        <f>F10*characterization!$J$17 + G10*characterization!$J$15</f>
+        <f>F10*characterization!$L$17 + G10*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L10" s="7">
@@ -3531,7 +4029,7 @@
         </is>
       </c>
       <c r="I11" s="7">
-        <f>F11*characterization!$D$17 + G11*characterization!$D$15</f>
+        <f>F11*characterization!$B$17 + G11*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J11" s="7">
@@ -3539,7 +4037,7 @@
         <v/>
       </c>
       <c r="K11" s="7">
-        <f>F11*characterization!$J$17 + G11*characterization!$J$15</f>
+        <f>F11*characterization!$L$17 + G11*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L11" s="7">
@@ -3606,7 +4104,7 @@
         </is>
       </c>
       <c r="I12" s="7">
-        <f>F12*characterization!$D$17 + G12*characterization!$D$15</f>
+        <f>F12*characterization!$B$17 + G12*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J12" s="7">
@@ -3614,7 +4112,7 @@
         <v/>
       </c>
       <c r="K12" s="7">
-        <f>F12*characterization!$J$17 + G12*characterization!$J$15</f>
+        <f>F12*characterization!$L$17 + G12*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L12" s="7">
@@ -3688,7 +4186,7 @@
         </is>
       </c>
       <c r="I14" s="7">
-        <f>F14*characterization!$D$17 + G14*characterization!$D$15</f>
+        <f>F14*characterization!$B$17 + G14*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J14" s="7">
@@ -3696,7 +4194,7 @@
         <v/>
       </c>
       <c r="K14" s="7">
-        <f>F14*characterization!$J$17 + G14*characterization!$J$15</f>
+        <f>F14*characterization!$L$17 + G14*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L14" s="7">
@@ -3763,7 +4261,7 @@
         </is>
       </c>
       <c r="I15" s="7">
-        <f>F15*characterization!$D$17 + G15*characterization!$D$15</f>
+        <f>F15*characterization!$B$17 + G15*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J15" s="7">
@@ -3771,7 +4269,7 @@
         <v/>
       </c>
       <c r="K15" s="7">
-        <f>F15*characterization!$J$17 + G15*characterization!$J$15</f>
+        <f>F15*characterization!$L$17 + G15*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L15" s="7">
@@ -3838,7 +4336,7 @@
         </is>
       </c>
       <c r="I16" s="7">
-        <f>F16*characterization!$D$17 + G16*characterization!$D$15</f>
+        <f>F16*characterization!$B$17 + G16*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J16" s="7">
@@ -3846,7 +4344,7 @@
         <v/>
       </c>
       <c r="K16" s="7">
-        <f>F16*characterization!$J$17 + G16*characterization!$J$15</f>
+        <f>F16*characterization!$L$17 + G16*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L16" s="7">
@@ -3913,7 +4411,7 @@
         </is>
       </c>
       <c r="I17" s="7">
-        <f>F17*characterization!$D$17 + G17*characterization!$D$15</f>
+        <f>F17*characterization!$B$17 + G17*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J17" s="7">
@@ -3921,7 +4419,7 @@
         <v/>
       </c>
       <c r="K17" s="7">
-        <f>F17*characterization!$J$17 + G17*characterization!$J$15</f>
+        <f>F17*characterization!$L$17 + G17*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L17" s="7">
@@ -3988,7 +4486,7 @@
         </is>
       </c>
       <c r="I18" s="7">
-        <f>F18*characterization!$D$17 + G18*characterization!$D$15</f>
+        <f>F18*characterization!$B$17 + G18*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J18" s="7">
@@ -3996,7 +4494,7 @@
         <v/>
       </c>
       <c r="K18" s="7">
-        <f>F18*characterization!$J$17 + G18*characterization!$J$15</f>
+        <f>F18*characterization!$L$17 + G18*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L18" s="7">
@@ -4063,7 +4561,7 @@
         </is>
       </c>
       <c r="I19" s="7">
-        <f>F19*characterization!$D$17 + G19*characterization!$D$15</f>
+        <f>F19*characterization!$B$17 + G19*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J19" s="7">
@@ -4071,7 +4569,7 @@
         <v/>
       </c>
       <c r="K19" s="7">
-        <f>F19*characterization!$J$17 + G19*characterization!$J$15</f>
+        <f>F19*characterization!$L$17 + G19*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L19" s="7">
@@ -4138,7 +4636,7 @@
         </is>
       </c>
       <c r="I20" s="7">
-        <f>F20*characterization!$D$17 + G20*characterization!$D$15</f>
+        <f>F20*characterization!$B$17 + G20*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J20" s="7">
@@ -4146,7 +4644,7 @@
         <v/>
       </c>
       <c r="K20" s="7">
-        <f>F20*characterization!$J$17 + G20*characterization!$J$15</f>
+        <f>F20*characterization!$L$17 + G20*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L20" s="7">
@@ -4213,7 +4711,7 @@
         </is>
       </c>
       <c r="I21" s="7">
-        <f>F21*characterization!$D$17 + G21*characterization!$D$15</f>
+        <f>F21*characterization!$B$17 + G21*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J21" s="7">
@@ -4221,7 +4719,7 @@
         <v/>
       </c>
       <c r="K21" s="7">
-        <f>F21*characterization!$J$17 + G21*characterization!$J$15</f>
+        <f>F21*characterization!$L$17 + G21*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L21" s="7">
@@ -4288,7 +4786,7 @@
         </is>
       </c>
       <c r="I22" s="7">
-        <f>F22*characterization!$D$17 + G22*characterization!$D$15</f>
+        <f>F22*characterization!$B$17 + G22*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J22" s="7">
@@ -4296,7 +4794,7 @@
         <v/>
       </c>
       <c r="K22" s="7">
-        <f>F22*characterization!$J$17 + G22*characterization!$J$15</f>
+        <f>F22*characterization!$L$17 + G22*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L22" s="7">
@@ -4370,7 +4868,7 @@
         </is>
       </c>
       <c r="I24" s="7">
-        <f>F24*characterization!$D$17 + G24*characterization!$D$15</f>
+        <f>F24*characterization!$B$17 + G24*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J24" s="7">
@@ -4378,7 +4876,7 @@
         <v/>
       </c>
       <c r="K24" s="7">
-        <f>F24*characterization!$J$17 + G24*characterization!$J$15</f>
+        <f>F24*characterization!$L$17 + G24*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L24" s="7">
@@ -4445,7 +4943,7 @@
         </is>
       </c>
       <c r="I25" s="7">
-        <f>F25*characterization!$D$17 + G25*characterization!$D$15</f>
+        <f>F25*characterization!$B$17 + G25*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J25" s="7">
@@ -4453,7 +4951,7 @@
         <v/>
       </c>
       <c r="K25" s="7">
-        <f>F25*characterization!$J$17 + G25*characterization!$J$15</f>
+        <f>F25*characterization!$L$17 + G25*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L25" s="7">
@@ -4520,7 +5018,7 @@
         </is>
       </c>
       <c r="I26" s="7">
-        <f>F26*characterization!$D$17 + G26*characterization!$D$15</f>
+        <f>F26*characterization!$B$17 + G26*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J26" s="7">
@@ -4528,7 +5026,7 @@
         <v/>
       </c>
       <c r="K26" s="7">
-        <f>F26*characterization!$J$17 + G26*characterization!$J$15</f>
+        <f>F26*characterization!$L$17 + G26*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L26" s="7">
@@ -4595,7 +5093,7 @@
         </is>
       </c>
       <c r="I27" s="7">
-        <f>F27*characterization!$D$17 + G27*characterization!$D$15</f>
+        <f>F27*characterization!$B$17 + G27*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J27" s="7">
@@ -4603,7 +5101,7 @@
         <v/>
       </c>
       <c r="K27" s="7">
-        <f>F27*characterization!$J$17 + G27*characterization!$J$15</f>
+        <f>F27*characterization!$L$17 + G27*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L27" s="7">
@@ -4670,7 +5168,7 @@
         </is>
       </c>
       <c r="I28" s="7">
-        <f>F28*characterization!$D$17 + G28*characterization!$D$15</f>
+        <f>F28*characterization!$B$17 + G28*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J28" s="7">
@@ -4678,7 +5176,7 @@
         <v/>
       </c>
       <c r="K28" s="7">
-        <f>F28*characterization!$J$17 + G28*characterization!$J$15</f>
+        <f>F28*characterization!$L$17 + G28*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L28" s="7">
@@ -4745,7 +5243,7 @@
         </is>
       </c>
       <c r="I29" s="7">
-        <f>F29*characterization!$D$17 + G29*characterization!$D$15</f>
+        <f>F29*characterization!$B$17 + G29*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J29" s="7">
@@ -4753,7 +5251,7 @@
         <v/>
       </c>
       <c r="K29" s="7">
-        <f>F29*characterization!$J$17 + G29*characterization!$J$15</f>
+        <f>F29*characterization!$L$17 + G29*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L29" s="7">
@@ -4820,7 +5318,7 @@
         </is>
       </c>
       <c r="I30" s="7">
-        <f>F30*characterization!$D$17 + G30*characterization!$D$15</f>
+        <f>F30*characterization!$B$17 + G30*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J30" s="7">
@@ -4828,7 +5326,7 @@
         <v/>
       </c>
       <c r="K30" s="7">
-        <f>F30*characterization!$J$17 + G30*characterization!$J$15</f>
+        <f>F30*characterization!$L$17 + G30*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L30" s="7">
@@ -4895,7 +5393,7 @@
         </is>
       </c>
       <c r="I31" s="7">
-        <f>F31*characterization!$D$17 + G31*characterization!$D$15</f>
+        <f>F31*characterization!$B$17 + G31*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J31" s="7">
@@ -4903,7 +5401,7 @@
         <v/>
       </c>
       <c r="K31" s="7">
-        <f>F31*characterization!$J$17 + G31*characterization!$J$15</f>
+        <f>F31*characterization!$L$17 + G31*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L31" s="7">
@@ -4970,7 +5468,7 @@
         </is>
       </c>
       <c r="I32" s="7">
-        <f>F32*characterization!$D$17 + G32*characterization!$D$15</f>
+        <f>F32*characterization!$B$17 + G32*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J32" s="7">
@@ -4978,7 +5476,7 @@
         <v/>
       </c>
       <c r="K32" s="7">
-        <f>F32*characterization!$J$17 + G32*characterization!$J$15</f>
+        <f>F32*characterization!$L$17 + G32*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L32" s="7">
@@ -5052,7 +5550,7 @@
         </is>
       </c>
       <c r="I34" s="7">
-        <f>F34*characterization!$D$17 + G34*characterization!$D$15</f>
+        <f>F34*characterization!$B$17 + G34*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J34" s="7">
@@ -5060,7 +5558,7 @@
         <v/>
       </c>
       <c r="K34" s="7">
-        <f>F34*characterization!$J$17 + G34*characterization!$J$15</f>
+        <f>F34*characterization!$L$17 + G34*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L34" s="7">
@@ -5127,7 +5625,7 @@
         </is>
       </c>
       <c r="I35" s="7">
-        <f>F35*characterization!$D$17 + G35*characterization!$D$15</f>
+        <f>F35*characterization!$B$17 + G35*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J35" s="7">
@@ -5135,7 +5633,7 @@
         <v/>
       </c>
       <c r="K35" s="7">
-        <f>F35*characterization!$J$17 + G35*characterization!$J$15</f>
+        <f>F35*characterization!$L$17 + G35*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L35" s="7">
@@ -5202,7 +5700,7 @@
         </is>
       </c>
       <c r="I36" s="7">
-        <f>F36*characterization!$D$17 + G36*characterization!$D$15</f>
+        <f>F36*characterization!$B$17 + G36*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J36" s="7">
@@ -5210,7 +5708,7 @@
         <v/>
       </c>
       <c r="K36" s="7">
-        <f>F36*characterization!$J$17 + G36*characterization!$J$15</f>
+        <f>F36*characterization!$L$17 + G36*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L36" s="7">
@@ -5277,7 +5775,7 @@
         </is>
       </c>
       <c r="I37" s="7">
-        <f>F37*characterization!$D$17 + G37*characterization!$D$15</f>
+        <f>F37*characterization!$B$17 + G37*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J37" s="7">
@@ -5285,7 +5783,7 @@
         <v/>
       </c>
       <c r="K37" s="7">
-        <f>F37*characterization!$J$17 + G37*characterization!$J$15</f>
+        <f>F37*characterization!$L$17 + G37*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L37" s="7">
@@ -5356,7 +5854,7 @@
         </is>
       </c>
       <c r="I38" s="7">
-        <f>F38*characterization!$D$17 + G38*characterization!$D$15</f>
+        <f>F38*characterization!$B$17 + G38*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J38" s="7">
@@ -5364,7 +5862,7 @@
         <v/>
       </c>
       <c r="K38" s="7">
-        <f>F38*characterization!$J$17 + G38*characterization!$J$15</f>
+        <f>F38*characterization!$L$17 + G38*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L38" s="7">
@@ -5435,7 +5933,7 @@
         </is>
       </c>
       <c r="I39" s="7">
-        <f>F39*characterization!$D$17 + G39*characterization!$D$15</f>
+        <f>F39*characterization!$B$17 + G39*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J39" s="7">
@@ -5443,7 +5941,7 @@
         <v/>
       </c>
       <c r="K39" s="7">
-        <f>F39*characterization!$J$17 + G39*characterization!$J$15</f>
+        <f>F39*characterization!$L$17 + G39*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L39" s="7">
@@ -5514,7 +6012,7 @@
         </is>
       </c>
       <c r="I40" s="7">
-        <f>F40*characterization!$D$17 + G40*characterization!$D$15</f>
+        <f>F40*characterization!$B$17 + G40*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J40" s="7">
@@ -5522,7 +6020,7 @@
         <v/>
       </c>
       <c r="K40" s="7">
-        <f>F40*characterization!$J$17 + G40*characterization!$J$15</f>
+        <f>F40*characterization!$L$17 + G40*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L40" s="7">
@@ -5589,7 +6087,7 @@
         </is>
       </c>
       <c r="I41" s="7">
-        <f>F41*characterization!$D$17 + G41*characterization!$D$15</f>
+        <f>F41*characterization!$B$17 + G41*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J41" s="7">
@@ -5597,7 +6095,7 @@
         <v/>
       </c>
       <c r="K41" s="7">
-        <f>F41*characterization!$J$17 + G41*characterization!$J$15</f>
+        <f>F41*characterization!$L$17 + G41*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L41" s="7">
@@ -5668,7 +6166,7 @@
         </is>
       </c>
       <c r="I42" s="7">
-        <f>F42*characterization!$D$17 + G42*characterization!$D$15</f>
+        <f>F42*characterization!$B$17 + G42*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J42" s="7">
@@ -5676,7 +6174,7 @@
         <v/>
       </c>
       <c r="K42" s="7">
-        <f>F42*characterization!$J$17 + G42*characterization!$J$15</f>
+        <f>F42*characterization!$L$17 + G42*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L42" s="7">
@@ -5743,7 +6241,7 @@
         </is>
       </c>
       <c r="I43" s="7">
-        <f>F43*characterization!$D$17 + G43*characterization!$D$15</f>
+        <f>F43*characterization!$B$17 + G43*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J43" s="7">
@@ -5751,7 +6249,7 @@
         <v/>
       </c>
       <c r="K43" s="7">
-        <f>F43*characterization!$J$17 + G43*characterization!$J$15</f>
+        <f>F43*characterization!$L$17 + G43*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L43" s="7">
@@ -5818,7 +6316,7 @@
         </is>
       </c>
       <c r="I44" s="7">
-        <f>F44*characterization!$D$17 + G44*characterization!$D$15</f>
+        <f>F44*characterization!$B$17 + G44*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J44" s="7">
@@ -5826,7 +6324,7 @@
         <v/>
       </c>
       <c r="K44" s="7">
-        <f>F44*characterization!$J$17 + G44*characterization!$J$15</f>
+        <f>F44*characterization!$L$17 + G44*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L44" s="7">
@@ -5900,7 +6398,7 @@
         </is>
       </c>
       <c r="I46" s="7">
-        <f>F46*characterization!$D$17 + G46*characterization!$D$15</f>
+        <f>F46*characterization!$B$17 + G46*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J46" s="7">
@@ -5908,7 +6406,7 @@
         <v/>
       </c>
       <c r="K46" s="7">
-        <f>F46*characterization!$J$17 + G46*characterization!$J$15</f>
+        <f>F46*characterization!$L$17 + G46*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L46" s="7">
@@ -5975,7 +6473,7 @@
         </is>
       </c>
       <c r="I47" s="7">
-        <f>F47*characterization!$D$17 + G47*characterization!$D$15</f>
+        <f>F47*characterization!$B$17 + G47*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J47" s="7">
@@ -5983,7 +6481,7 @@
         <v/>
       </c>
       <c r="K47" s="7">
-        <f>F47*characterization!$J$17 + G47*characterization!$J$15</f>
+        <f>F47*characterization!$L$17 + G47*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L47" s="7">
@@ -6050,7 +6548,7 @@
         </is>
       </c>
       <c r="I48" s="7">
-        <f>F48*characterization!$D$17 + G48*characterization!$D$15</f>
+        <f>F48*characterization!$B$17 + G48*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J48" s="7">
@@ -6058,7 +6556,7 @@
         <v/>
       </c>
       <c r="K48" s="7">
-        <f>F48*characterization!$J$17 + G48*characterization!$J$15</f>
+        <f>F48*characterization!$L$17 + G48*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L48" s="7">
@@ -6125,7 +6623,7 @@
         </is>
       </c>
       <c r="I49" s="7">
-        <f>F49*characterization!$D$17 + G49*characterization!$D$15</f>
+        <f>F49*characterization!$B$17 + G49*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J49" s="7">
@@ -6133,7 +6631,7 @@
         <v/>
       </c>
       <c r="K49" s="7">
-        <f>F49*characterization!$J$17 + G49*characterization!$J$15</f>
+        <f>F49*characterization!$L$17 + G49*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L49" s="7">
@@ -6200,7 +6698,7 @@
         </is>
       </c>
       <c r="I50" s="7">
-        <f>F50*characterization!$D$17 + G50*characterization!$D$15</f>
+        <f>F50*characterization!$B$17 + G50*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J50" s="7">
@@ -6208,7 +6706,7 @@
         <v/>
       </c>
       <c r="K50" s="7">
-        <f>F50*characterization!$J$17 + G50*characterization!$J$15</f>
+        <f>F50*characterization!$L$17 + G50*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L50" s="7">
@@ -6282,7 +6780,7 @@
         </is>
       </c>
       <c r="I52" s="7">
-        <f>F52*characterization!$D$17 + G52*characterization!$D$15</f>
+        <f>F52*characterization!$B$17 + G52*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J52" s="7">
@@ -6290,7 +6788,7 @@
         <v/>
       </c>
       <c r="K52" s="7">
-        <f>F52*characterization!$J$17 + G52*characterization!$J$15</f>
+        <f>F52*characterization!$L$17 + G52*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L52" s="7">
@@ -6357,7 +6855,7 @@
         </is>
       </c>
       <c r="I53" s="7">
-        <f>F53*characterization!$D$17 + G53*characterization!$D$15</f>
+        <f>F53*characterization!$B$17 + G53*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J53" s="7">
@@ -6365,7 +6863,7 @@
         <v/>
       </c>
       <c r="K53" s="7">
-        <f>F53*characterization!$J$17 + G53*characterization!$J$15</f>
+        <f>F53*characterization!$L$17 + G53*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L53" s="7">
@@ -6432,7 +6930,7 @@
         </is>
       </c>
       <c r="I54" s="7">
-        <f>F54*characterization!$D$17 + G54*characterization!$D$15</f>
+        <f>F54*characterization!$B$17 + G54*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J54" s="7">
@@ -6440,7 +6938,7 @@
         <v/>
       </c>
       <c r="K54" s="7">
-        <f>F54*characterization!$J$17 + G54*characterization!$J$15</f>
+        <f>F54*characterization!$L$17 + G54*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L54" s="7">
@@ -6507,7 +7005,7 @@
         </is>
       </c>
       <c r="I55" s="7">
-        <f>F55*characterization!$D$17 + G55*characterization!$D$15</f>
+        <f>F55*characterization!$B$17 + G55*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J55" s="7">
@@ -6515,7 +7013,7 @@
         <v/>
       </c>
       <c r="K55" s="7">
-        <f>F55*characterization!$J$17 + G55*characterization!$J$15</f>
+        <f>F55*characterization!$L$17 + G55*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L55" s="7">
@@ -6582,7 +7080,7 @@
         </is>
       </c>
       <c r="I56" s="7">
-        <f>F56*characterization!$D$17 + G56*characterization!$D$15</f>
+        <f>F56*characterization!$B$17 + G56*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J56" s="7">
@@ -6590,7 +7088,7 @@
         <v/>
       </c>
       <c r="K56" s="7">
-        <f>F56*characterization!$J$17 + G56*characterization!$J$15</f>
+        <f>F56*characterization!$L$17 + G56*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L56" s="7">
@@ -6657,7 +7155,7 @@
         </is>
       </c>
       <c r="I57" s="7">
-        <f>F57*characterization!$D$17 + G57*characterization!$D$15</f>
+        <f>F57*characterization!$B$17 + G57*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J57" s="7">
@@ -6665,7 +7163,7 @@
         <v/>
       </c>
       <c r="K57" s="7">
-        <f>F57*characterization!$J$17 + G57*characterization!$J$15</f>
+        <f>F57*characterization!$L$17 + G57*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L57" s="7">
@@ -6732,7 +7230,7 @@
         </is>
       </c>
       <c r="I58" s="7">
-        <f>F58*characterization!$D$17 + G58*characterization!$D$15</f>
+        <f>F58*characterization!$B$17 + G58*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J58" s="7">
@@ -6740,7 +7238,7 @@
         <v/>
       </c>
       <c r="K58" s="7">
-        <f>F58*characterization!$J$17 + G58*characterization!$J$15</f>
+        <f>F58*characterization!$L$17 + G58*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L58" s="7">
@@ -6811,7 +7309,7 @@
         </is>
       </c>
       <c r="I59" s="7">
-        <f>F59*characterization!$D$17 + G59*characterization!$D$15</f>
+        <f>F59*characterization!$B$17 + G59*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J59" s="7">
@@ -6819,7 +7317,7 @@
         <v/>
       </c>
       <c r="K59" s="7">
-        <f>F59*characterization!$J$17 + G59*characterization!$J$15</f>
+        <f>F59*characterization!$L$17 + G59*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L59" s="7">
@@ -6890,7 +7388,7 @@
         </is>
       </c>
       <c r="I60" s="7">
-        <f>F60*characterization!$D$17 + G60*characterization!$D$15</f>
+        <f>F60*characterization!$B$17 + G60*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J60" s="7">
@@ -6898,7 +7396,7 @@
         <v/>
       </c>
       <c r="K60" s="7">
-        <f>F60*characterization!$J$17 + G60*characterization!$J$15</f>
+        <f>F60*characterization!$L$17 + G60*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L60" s="7">
@@ -6969,7 +7467,7 @@
         </is>
       </c>
       <c r="I61" s="7">
-        <f>F61*characterization!$D$17 + G61*characterization!$D$15</f>
+        <f>F61*characterization!$B$17 + G61*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J61" s="7">
@@ -6977,7 +7475,7 @@
         <v/>
       </c>
       <c r="K61" s="7">
-        <f>F61*characterization!$J$17 + G61*characterization!$J$15</f>
+        <f>F61*characterization!$L$17 + G61*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L61" s="7">
@@ -7048,7 +7546,7 @@
         </is>
       </c>
       <c r="I62" s="7">
-        <f>F62*characterization!$D$17 + G62*characterization!$D$15</f>
+        <f>F62*characterization!$B$17 + G62*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J62" s="7">
@@ -7056,7 +7554,7 @@
         <v/>
       </c>
       <c r="K62" s="7">
-        <f>F62*characterization!$J$17 + G62*characterization!$J$15</f>
+        <f>F62*characterization!$L$17 + G62*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L62" s="7">
@@ -7127,7 +7625,7 @@
         </is>
       </c>
       <c r="I63" s="7">
-        <f>F63*characterization!$D$17 + G63*characterization!$D$15</f>
+        <f>F63*characterization!$B$17 + G63*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J63" s="7">
@@ -7135,7 +7633,7 @@
         <v/>
       </c>
       <c r="K63" s="7">
-        <f>F63*characterization!$J$17 + G63*characterization!$J$15</f>
+        <f>F63*characterization!$L$17 + G63*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L63" s="7">
@@ -7209,7 +7707,7 @@
         </is>
       </c>
       <c r="I65" s="7">
-        <f>F65*characterization!$D$17 + G65*characterization!$D$15</f>
+        <f>F65*characterization!$B$17 + G65*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J65" s="7">
@@ -7217,7 +7715,7 @@
         <v/>
       </c>
       <c r="K65" s="7">
-        <f>F65*characterization!$J$17 + G65*characterization!$J$15</f>
+        <f>F65*characterization!$L$17 + G65*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L65" s="7">
@@ -7284,7 +7782,7 @@
         </is>
       </c>
       <c r="I66" s="7">
-        <f>F66*characterization!$D$17 + G66*characterization!$D$15</f>
+        <f>F66*characterization!$B$17 + G66*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J66" s="7">
@@ -7292,7 +7790,7 @@
         <v/>
       </c>
       <c r="K66" s="7">
-        <f>F66*characterization!$J$17 + G66*characterization!$J$15</f>
+        <f>F66*characterization!$L$17 + G66*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L66" s="7">
@@ -7359,7 +7857,7 @@
         </is>
       </c>
       <c r="I67" s="7">
-        <f>F67*characterization!$D$17 + G67*characterization!$D$15</f>
+        <f>F67*characterization!$B$17 + G67*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J67" s="7">
@@ -7367,7 +7865,7 @@
         <v/>
       </c>
       <c r="K67" s="7">
-        <f>F67*characterization!$J$17 + G67*characterization!$J$15</f>
+        <f>F67*characterization!$L$17 + G67*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L67" s="7">
@@ -7434,7 +7932,7 @@
         </is>
       </c>
       <c r="I68" s="7">
-        <f>F68*characterization!$D$17 + G68*characterization!$D$15</f>
+        <f>F68*characterization!$B$17 + G68*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J68" s="7">
@@ -7442,7 +7940,7 @@
         <v/>
       </c>
       <c r="K68" s="7">
-        <f>F68*characterization!$J$17 + G68*characterization!$J$15</f>
+        <f>F68*characterization!$L$17 + G68*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L68" s="7">
@@ -7509,7 +8007,7 @@
         </is>
       </c>
       <c r="I69" s="7">
-        <f>F69*characterization!$D$17 + G69*characterization!$D$15</f>
+        <f>F69*characterization!$B$17 + G69*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J69" s="7">
@@ -7517,7 +8015,7 @@
         <v/>
       </c>
       <c r="K69" s="7">
-        <f>F69*characterization!$J$17 + G69*characterization!$J$15</f>
+        <f>F69*characterization!$L$17 + G69*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L69" s="7">
@@ -7584,7 +8082,7 @@
         </is>
       </c>
       <c r="I70" s="7">
-        <f>F70*characterization!$D$17 + G70*characterization!$D$15</f>
+        <f>F70*characterization!$B$17 + G70*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J70" s="7">
@@ -7592,7 +8090,7 @@
         <v/>
       </c>
       <c r="K70" s="7">
-        <f>F70*characterization!$J$17 + G70*characterization!$J$15</f>
+        <f>F70*characterization!$L$17 + G70*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L70" s="7">
@@ -7659,7 +8157,7 @@
         </is>
       </c>
       <c r="I71" s="7">
-        <f>F71*characterization!$D$17 + G71*characterization!$D$15</f>
+        <f>F71*characterization!$B$17 + G71*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J71" s="7">
@@ -7667,7 +8165,7 @@
         <v/>
       </c>
       <c r="K71" s="7">
-        <f>F71*characterization!$J$17 + G71*characterization!$J$15</f>
+        <f>F71*characterization!$L$17 + G71*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L71" s="7">
@@ -7734,7 +8232,7 @@
         </is>
       </c>
       <c r="I72" s="7">
-        <f>F72*characterization!$D$17 + G72*characterization!$D$15</f>
+        <f>F72*characterization!$B$17 + G72*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J72" s="7">
@@ -7742,7 +8240,7 @@
         <v/>
       </c>
       <c r="K72" s="7">
-        <f>F72*characterization!$J$17 + G72*characterization!$J$15</f>
+        <f>F72*characterization!$L$17 + G72*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L72" s="7">
@@ -7809,7 +8307,7 @@
         </is>
       </c>
       <c r="I73" s="7">
-        <f>F73*characterization!$D$17 + G73*characterization!$D$15</f>
+        <f>F73*characterization!$B$17 + G73*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J73" s="7">
@@ -7817,7 +8315,7 @@
         <v/>
       </c>
       <c r="K73" s="7">
-        <f>F73*characterization!$J$17 + G73*characterization!$J$15</f>
+        <f>F73*characterization!$L$17 + G73*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L73" s="7">
@@ -7884,7 +8382,7 @@
         </is>
       </c>
       <c r="I74" s="7">
-        <f>F74*characterization!$D$17 + G74*characterization!$D$15</f>
+        <f>F74*characterization!$B$17 + G74*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J74" s="7">
@@ -7892,7 +8390,7 @@
         <v/>
       </c>
       <c r="K74" s="7">
-        <f>F74*characterization!$J$17 + G74*characterization!$J$15</f>
+        <f>F74*characterization!$L$17 + G74*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L74" s="7">
@@ -7959,7 +8457,7 @@
         </is>
       </c>
       <c r="I75" s="7">
-        <f>F75*characterization!$D$17 + G75*characterization!$D$15</f>
+        <f>F75*characterization!$B$17 + G75*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J75" s="7">
@@ -7967,7 +8465,7 @@
         <v/>
       </c>
       <c r="K75" s="7">
-        <f>F75*characterization!$J$17 + G75*characterization!$J$15</f>
+        <f>F75*characterization!$L$17 + G75*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L75" s="7">
@@ -8041,7 +8539,7 @@
         </is>
       </c>
       <c r="I77" s="7">
-        <f>F77*characterization!$D$17 + G77*characterization!$D$15</f>
+        <f>F77*characterization!$B$17 + G77*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J77" s="7">
@@ -8049,7 +8547,7 @@
         <v/>
       </c>
       <c r="K77" s="7">
-        <f>F77*characterization!$J$17 + G77*characterization!$J$15</f>
+        <f>F77*characterization!$L$17 + G77*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L77" s="7">
@@ -8116,7 +8614,7 @@
         </is>
       </c>
       <c r="I78" s="7">
-        <f>F78*characterization!$D$17 + G78*characterization!$D$15</f>
+        <f>F78*characterization!$B$17 + G78*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J78" s="7">
@@ -8124,7 +8622,7 @@
         <v/>
       </c>
       <c r="K78" s="7">
-        <f>F78*characterization!$J$17 + G78*characterization!$J$15</f>
+        <f>F78*characterization!$L$17 + G78*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L78" s="7">
@@ -8191,7 +8689,7 @@
         </is>
       </c>
       <c r="I79" s="7">
-        <f>F79*characterization!$D$17 + G79*characterization!$D$15</f>
+        <f>F79*characterization!$B$17 + G79*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J79" s="7">
@@ -8199,7 +8697,7 @@
         <v/>
       </c>
       <c r="K79" s="7">
-        <f>F79*characterization!$J$17 + G79*characterization!$J$15</f>
+        <f>F79*characterization!$L$17 + G79*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L79" s="7">
@@ -8266,7 +8764,7 @@
         </is>
       </c>
       <c r="I80" s="7">
-        <f>F80*characterization!$D$17 + G80*characterization!$D$15</f>
+        <f>F80*characterization!$B$17 + G80*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J80" s="7">
@@ -8274,7 +8772,7 @@
         <v/>
       </c>
       <c r="K80" s="7">
-        <f>F80*characterization!$J$17 + G80*characterization!$J$15</f>
+        <f>F80*characterization!$L$17 + G80*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L80" s="7">
@@ -8341,7 +8839,7 @@
         </is>
       </c>
       <c r="I81" s="7">
-        <f>F81*characterization!$D$17 + G81*characterization!$D$15</f>
+        <f>F81*characterization!$B$17 + G81*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J81" s="7">
@@ -8349,7 +8847,7 @@
         <v/>
       </c>
       <c r="K81" s="7">
-        <f>F81*characterization!$J$17 + G81*characterization!$J$15</f>
+        <f>F81*characterization!$L$17 + G81*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L81" s="7">
@@ -8416,7 +8914,7 @@
         </is>
       </c>
       <c r="I82" s="7">
-        <f>F82*characterization!$D$17 + G82*characterization!$D$15</f>
+        <f>F82*characterization!$B$17 + G82*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J82" s="7">
@@ -8424,7 +8922,7 @@
         <v/>
       </c>
       <c r="K82" s="7">
-        <f>F82*characterization!$J$17 + G82*characterization!$J$15</f>
+        <f>F82*characterization!$L$17 + G82*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L82" s="7">
@@ -8495,7 +8993,7 @@
         </is>
       </c>
       <c r="I83" s="7">
-        <f>F83*characterization!$D$17 + G83*characterization!$D$15</f>
+        <f>F83*characterization!$B$17 + G83*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J83" s="7">
@@ -8503,7 +9001,7 @@
         <v/>
       </c>
       <c r="K83" s="7">
-        <f>F83*characterization!$J$17 + G83*characterization!$J$15</f>
+        <f>F83*characterization!$L$17 + G83*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L83" s="7">
@@ -8574,7 +9072,7 @@
         </is>
       </c>
       <c r="I84" s="7">
-        <f>F84*characterization!$D$17 + G84*characterization!$D$15</f>
+        <f>F84*characterization!$B$17 + G84*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J84" s="7">
@@ -8582,7 +9080,7 @@
         <v/>
       </c>
       <c r="K84" s="7">
-        <f>F84*characterization!$J$17 + G84*characterization!$J$15</f>
+        <f>F84*characterization!$L$17 + G84*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L84" s="7">
@@ -8653,7 +9151,7 @@
         </is>
       </c>
       <c r="I85" s="7">
-        <f>F85*characterization!$D$17 + G85*characterization!$D$15</f>
+        <f>F85*characterization!$B$17 + G85*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J85" s="7">
@@ -8661,7 +9159,7 @@
         <v/>
       </c>
       <c r="K85" s="7">
-        <f>F85*characterization!$J$17 + G85*characterization!$J$15</f>
+        <f>F85*characterization!$L$17 + G85*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L85" s="7">
@@ -8732,7 +9230,7 @@
         </is>
       </c>
       <c r="I86" s="7">
-        <f>F86*characterization!$D$17 + G86*characterization!$D$15</f>
+        <f>F86*characterization!$B$17 + G86*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J86" s="7">
@@ -8740,7 +9238,7 @@
         <v/>
       </c>
       <c r="K86" s="7">
-        <f>F86*characterization!$J$17 + G86*characterization!$J$15</f>
+        <f>F86*characterization!$L$17 + G86*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L86" s="7">
@@ -8811,7 +9309,7 @@
         </is>
       </c>
       <c r="I87" s="7">
-        <f>F87*characterization!$D$17 + G87*characterization!$D$15</f>
+        <f>F87*characterization!$B$17 + G87*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J87" s="7">
@@ -8819,7 +9317,7 @@
         <v/>
       </c>
       <c r="K87" s="7">
-        <f>F87*characterization!$J$17 + G87*characterization!$J$15</f>
+        <f>F87*characterization!$L$17 + G87*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L87" s="7">
@@ -8893,7 +9391,7 @@
         </is>
       </c>
       <c r="I89" s="7">
-        <f>F89*characterization!$D$17 + G89*characterization!$D$15</f>
+        <f>F89*characterization!$B$17 + G89*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J89" s="7">
@@ -8901,7 +9399,7 @@
         <v/>
       </c>
       <c r="K89" s="7">
-        <f>F89*characterization!$J$17 + G89*characterization!$J$15</f>
+        <f>F89*characterization!$L$17 + G89*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L89" s="7">
@@ -8968,7 +9466,7 @@
         </is>
       </c>
       <c r="I90" s="7">
-        <f>F90*characterization!$D$17 + G90*characterization!$D$15</f>
+        <f>F90*characterization!$B$17 + G90*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J90" s="7">
@@ -8976,7 +9474,7 @@
         <v/>
       </c>
       <c r="K90" s="7">
-        <f>F90*characterization!$J$17 + G90*characterization!$J$15</f>
+        <f>F90*characterization!$L$17 + G90*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L90" s="7">
@@ -9043,7 +9541,7 @@
         </is>
       </c>
       <c r="I91" s="7">
-        <f>F91*characterization!$D$17 + G91*characterization!$D$15</f>
+        <f>F91*characterization!$B$17 + G91*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J91" s="7">
@@ -9051,7 +9549,7 @@
         <v/>
       </c>
       <c r="K91" s="7">
-        <f>F91*characterization!$J$17 + G91*characterization!$J$15</f>
+        <f>F91*characterization!$L$17 + G91*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L91" s="7">
@@ -9118,7 +9616,7 @@
         </is>
       </c>
       <c r="I92" s="7">
-        <f>F92*characterization!$D$17 + G92*characterization!$D$15</f>
+        <f>F92*characterization!$B$17 + G92*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J92" s="7">
@@ -9126,7 +9624,7 @@
         <v/>
       </c>
       <c r="K92" s="7">
-        <f>F92*characterization!$J$17 + G92*characterization!$J$15</f>
+        <f>F92*characterization!$L$17 + G92*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L92" s="7">
@@ -9193,7 +9691,7 @@
         </is>
       </c>
       <c r="I93" s="7">
-        <f>F93*characterization!$D$17 + G93*characterization!$D$15</f>
+        <f>F93*characterization!$B$17 + G93*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J93" s="7">
@@ -9201,7 +9699,7 @@
         <v/>
       </c>
       <c r="K93" s="7">
-        <f>F93*characterization!$J$17 + G93*characterization!$J$15</f>
+        <f>F93*characterization!$L$17 + G93*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L93" s="7">
@@ -9268,7 +9766,7 @@
         </is>
       </c>
       <c r="I94" s="7">
-        <f>F94*characterization!$D$17 + G94*characterization!$D$15</f>
+        <f>F94*characterization!$B$17 + G94*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J94" s="7">
@@ -9276,7 +9774,7 @@
         <v/>
       </c>
       <c r="K94" s="7">
-        <f>F94*characterization!$J$17 + G94*characterization!$J$15</f>
+        <f>F94*characterization!$L$17 + G94*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L94" s="7">
@@ -9343,7 +9841,7 @@
         </is>
       </c>
       <c r="I95" s="7">
-        <f>F95*characterization!$D$17 + G95*characterization!$D$15</f>
+        <f>F95*characterization!$B$17 + G95*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J95" s="7">
@@ -9351,7 +9849,7 @@
         <v/>
       </c>
       <c r="K95" s="7">
-        <f>F95*characterization!$J$17 + G95*characterization!$J$15</f>
+        <f>F95*characterization!$L$17 + G95*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L95" s="7">
@@ -9418,7 +9916,7 @@
         </is>
       </c>
       <c r="I96" s="7">
-        <f>F96*characterization!$D$17 + G96*characterization!$D$15</f>
+        <f>F96*characterization!$B$17 + G96*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J96" s="7">
@@ -9426,7 +9924,7 @@
         <v/>
       </c>
       <c r="K96" s="7">
-        <f>F96*characterization!$J$17 + G96*characterization!$J$15</f>
+        <f>F96*characterization!$L$17 + G96*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L96" s="7">
@@ -9493,7 +9991,7 @@
         </is>
       </c>
       <c r="I97" s="7">
-        <f>F97*characterization!$D$17 + G97*characterization!$D$15</f>
+        <f>F97*characterization!$B$17 + G97*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J97" s="7">
@@ -9501,7 +9999,7 @@
         <v/>
       </c>
       <c r="K97" s="7">
-        <f>F97*characterization!$J$17 + G97*characterization!$J$15</f>
+        <f>F97*characterization!$L$17 + G97*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L97" s="7">
@@ -9568,7 +10066,7 @@
         </is>
       </c>
       <c r="I98" s="7">
-        <f>F98*characterization!$D$17 + G98*characterization!$D$15</f>
+        <f>F98*characterization!$B$17 + G98*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J98" s="7">
@@ -9576,7 +10074,7 @@
         <v/>
       </c>
       <c r="K98" s="7">
-        <f>F98*characterization!$J$17 + G98*characterization!$J$15</f>
+        <f>F98*characterization!$L$17 + G98*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L98" s="7">
@@ -9643,7 +10141,7 @@
         </is>
       </c>
       <c r="I99" s="7">
-        <f>F99*characterization!$D$17 + G99*characterization!$D$15</f>
+        <f>F99*characterization!$B$17 + G99*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J99" s="7">
@@ -9651,7 +10149,7 @@
         <v/>
       </c>
       <c r="K99" s="7">
-        <f>F99*characterization!$J$17 + G99*characterization!$J$15</f>
+        <f>F99*characterization!$L$17 + G99*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L99" s="7">
@@ -9718,7 +10216,7 @@
         </is>
       </c>
       <c r="I100" s="7">
-        <f>F100*characterization!$D$17 + G100*characterization!$D$15</f>
+        <f>F100*characterization!$B$17 + G100*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J100" s="7">
@@ -9726,7 +10224,7 @@
         <v/>
       </c>
       <c r="K100" s="7">
-        <f>F100*characterization!$J$17 + G100*characterization!$J$15</f>
+        <f>F100*characterization!$L$17 + G100*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L100" s="7">
@@ -9793,7 +10291,7 @@
         </is>
       </c>
       <c r="I101" s="7">
-        <f>F101*characterization!$D$17 + G101*characterization!$D$15</f>
+        <f>F101*characterization!$B$17 + G101*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J101" s="7">
@@ -9801,7 +10299,7 @@
         <v/>
       </c>
       <c r="K101" s="7">
-        <f>F101*characterization!$J$17 + G101*characterization!$J$15</f>
+        <f>F101*characterization!$L$17 + G101*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L101" s="7">
@@ -9868,7 +10366,7 @@
         </is>
       </c>
       <c r="I102" s="7">
-        <f>F102*characterization!$D$17 + G102*characterization!$D$15</f>
+        <f>F102*characterization!$B$17 + G102*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J102" s="7">
@@ -9876,7 +10374,7 @@
         <v/>
       </c>
       <c r="K102" s="7">
-        <f>F102*characterization!$J$17 + G102*characterization!$J$15</f>
+        <f>F102*characterization!$L$17 + G102*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L102" s="7">
@@ -9950,7 +10448,7 @@
         </is>
       </c>
       <c r="I104" s="7">
-        <f>F104*characterization!$D$17 + G104*characterization!$D$15</f>
+        <f>F104*characterization!$B$17 + G104*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J104" s="7">
@@ -9958,7 +10456,7 @@
         <v/>
       </c>
       <c r="K104" s="7">
-        <f>F104*characterization!$J$17 + G104*characterization!$J$15</f>
+        <f>F104*characterization!$L$17 + G104*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L104" s="7">
@@ -10025,7 +10523,7 @@
         </is>
       </c>
       <c r="I105" s="7">
-        <f>F105*characterization!$D$17 + G105*characterization!$D$15</f>
+        <f>F105*characterization!$B$17 + G105*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J105" s="7">
@@ -10033,7 +10531,7 @@
         <v/>
       </c>
       <c r="K105" s="7">
-        <f>F105*characterization!$J$17 + G105*characterization!$J$15</f>
+        <f>F105*characterization!$L$17 + G105*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L105" s="7">
@@ -10100,7 +10598,7 @@
         </is>
       </c>
       <c r="I106" s="7">
-        <f>F106*characterization!$D$17 + G106*characterization!$D$15</f>
+        <f>F106*characterization!$B$17 + G106*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J106" s="7">
@@ -10108,7 +10606,7 @@
         <v/>
       </c>
       <c r="K106" s="7">
-        <f>F106*characterization!$J$17 + G106*characterization!$J$15</f>
+        <f>F106*characterization!$L$17 + G106*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L106" s="7">
@@ -10175,7 +10673,7 @@
         </is>
       </c>
       <c r="I107" s="7">
-        <f>F107*characterization!$D$17 + G107*characterization!$D$15</f>
+        <f>F107*characterization!$B$17 + G107*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J107" s="7">
@@ -10183,7 +10681,7 @@
         <v/>
       </c>
       <c r="K107" s="7">
-        <f>F107*characterization!$J$17 + G107*characterization!$J$15</f>
+        <f>F107*characterization!$L$17 + G107*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L107" s="7">
@@ -10250,7 +10748,7 @@
         </is>
       </c>
       <c r="I108" s="7">
-        <f>F108*characterization!$D$17 + G108*characterization!$D$15</f>
+        <f>F108*characterization!$B$17 + G108*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J108" s="7">
@@ -10258,7 +10756,7 @@
         <v/>
       </c>
       <c r="K108" s="7">
-        <f>F108*characterization!$J$17 + G108*characterization!$J$15</f>
+        <f>F108*characterization!$L$17 + G108*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L108" s="7">
@@ -10325,7 +10823,7 @@
         </is>
       </c>
       <c r="I109" s="7">
-        <f>F109*characterization!$D$17 + G109*characterization!$D$15</f>
+        <f>F109*characterization!$B$17 + G109*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J109" s="7">
@@ -10333,7 +10831,7 @@
         <v/>
       </c>
       <c r="K109" s="7">
-        <f>F109*characterization!$J$17 + G109*characterization!$J$15</f>
+        <f>F109*characterization!$L$17 + G109*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L109" s="7">
@@ -10400,7 +10898,7 @@
         </is>
       </c>
       <c r="I110" s="7">
-        <f>F110*characterization!$D$17 + G110*characterization!$D$15</f>
+        <f>F110*characterization!$B$17 + G110*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J110" s="7">
@@ -10408,7 +10906,7 @@
         <v/>
       </c>
       <c r="K110" s="7">
-        <f>F110*characterization!$J$17 + G110*characterization!$J$15</f>
+        <f>F110*characterization!$L$17 + G110*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L110" s="7">
@@ -10475,7 +10973,7 @@
         </is>
       </c>
       <c r="I111" s="7">
-        <f>F111*characterization!$D$17 + G111*characterization!$D$15</f>
+        <f>F111*characterization!$B$17 + G111*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J111" s="7">
@@ -10483,7 +10981,7 @@
         <v/>
       </c>
       <c r="K111" s="7">
-        <f>F111*characterization!$J$17 + G111*characterization!$J$15</f>
+        <f>F111*characterization!$L$17 + G111*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L111" s="7">
@@ -10554,7 +11052,7 @@
         </is>
       </c>
       <c r="I112" s="7">
-        <f>F112*characterization!$D$17 + G112*characterization!$D$15</f>
+        <f>F112*characterization!$B$17 + G112*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J112" s="7">
@@ -10562,7 +11060,7 @@
         <v/>
       </c>
       <c r="K112" s="7">
-        <f>F112*characterization!$J$17 + G112*characterization!$J$15</f>
+        <f>F112*characterization!$L$17 + G112*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L112" s="7">
@@ -10633,7 +11131,7 @@
         </is>
       </c>
       <c r="I113" s="7">
-        <f>F113*characterization!$D$17 + G113*characterization!$D$15</f>
+        <f>F113*characterization!$B$17 + G113*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J113" s="7">
@@ -10641,7 +11139,7 @@
         <v/>
       </c>
       <c r="K113" s="7">
-        <f>F113*characterization!$J$17 + G113*characterization!$J$15</f>
+        <f>F113*characterization!$L$17 + G113*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L113" s="7">
@@ -10708,7 +11206,7 @@
         </is>
       </c>
       <c r="I114" s="7">
-        <f>F114*characterization!$D$17 + G114*characterization!$D$15</f>
+        <f>F114*characterization!$B$17 + G114*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J114" s="7">
@@ -10716,7 +11214,7 @@
         <v/>
       </c>
       <c r="K114" s="7">
-        <f>F114*characterization!$J$17 + G114*characterization!$J$15</f>
+        <f>F114*characterization!$L$17 + G114*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L114" s="7">
@@ -10783,7 +11281,7 @@
         </is>
       </c>
       <c r="I115" s="7">
-        <f>F115*characterization!$D$17 + G115*characterization!$D$15</f>
+        <f>F115*characterization!$B$17 + G115*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J115" s="7">
@@ -10791,7 +11289,7 @@
         <v/>
       </c>
       <c r="K115" s="7">
-        <f>F115*characterization!$J$17 + G115*characterization!$J$15</f>
+        <f>F115*characterization!$L$17 + G115*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L115" s="7">
@@ -10858,7 +11356,7 @@
         </is>
       </c>
       <c r="I116" s="7">
-        <f>F116*characterization!$D$17 + G116*characterization!$D$15</f>
+        <f>F116*characterization!$B$17 + G116*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J116" s="7">
@@ -10866,7 +11364,7 @@
         <v/>
       </c>
       <c r="K116" s="7">
-        <f>F116*characterization!$J$17 + G116*characterization!$J$15</f>
+        <f>F116*characterization!$L$17 + G116*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L116" s="7">
@@ -10933,7 +11431,7 @@
         </is>
       </c>
       <c r="I117" s="7">
-        <f>F117*characterization!$D$17 + G117*characterization!$D$15</f>
+        <f>F117*characterization!$B$17 + G117*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J117" s="7">
@@ -10941,7 +11439,7 @@
         <v/>
       </c>
       <c r="K117" s="7">
-        <f>F117*characterization!$J$17 + G117*characterization!$J$15</f>
+        <f>F117*characterization!$L$17 + G117*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L117" s="7">
@@ -11015,7 +11513,7 @@
         </is>
       </c>
       <c r="I119" s="7">
-        <f>F119*characterization!$D$17 + G119*characterization!$D$15</f>
+        <f>F119*characterization!$B$17 + G119*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J119" s="7">
@@ -11023,7 +11521,7 @@
         <v/>
       </c>
       <c r="K119" s="7">
-        <f>F119*characterization!$J$17 + G119*characterization!$J$15</f>
+        <f>F119*characterization!$L$17 + G119*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L119" s="7">
@@ -11090,7 +11588,7 @@
         </is>
       </c>
       <c r="I120" s="7">
-        <f>F120*characterization!$D$17 + G120*characterization!$D$15</f>
+        <f>F120*characterization!$B$17 + G120*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J120" s="7">
@@ -11098,7 +11596,7 @@
         <v/>
       </c>
       <c r="K120" s="7">
-        <f>F120*characterization!$J$17 + G120*characterization!$J$15</f>
+        <f>F120*characterization!$L$17 + G120*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L120" s="7">
@@ -11165,7 +11663,7 @@
         </is>
       </c>
       <c r="I121" s="7">
-        <f>F121*characterization!$D$17 + G121*characterization!$D$15</f>
+        <f>F121*characterization!$B$17 + G121*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J121" s="7">
@@ -11173,7 +11671,7 @@
         <v/>
       </c>
       <c r="K121" s="7">
-        <f>F121*characterization!$J$17 + G121*characterization!$J$15</f>
+        <f>F121*characterization!$L$17 + G121*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L121" s="7">
@@ -11240,7 +11738,7 @@
         </is>
       </c>
       <c r="I122" s="7">
-        <f>F122*characterization!$D$17 + G122*characterization!$D$15</f>
+        <f>F122*characterization!$B$17 + G122*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J122" s="7">
@@ -11248,7 +11746,7 @@
         <v/>
       </c>
       <c r="K122" s="7">
-        <f>F122*characterization!$J$17 + G122*characterization!$J$15</f>
+        <f>F122*characterization!$L$17 + G122*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L122" s="7">
@@ -11315,7 +11813,7 @@
         </is>
       </c>
       <c r="I123" s="7">
-        <f>F123*characterization!$D$17 + G123*characterization!$D$15</f>
+        <f>F123*characterization!$B$17 + G123*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J123" s="7">
@@ -11323,7 +11821,7 @@
         <v/>
       </c>
       <c r="K123" s="7">
-        <f>F123*characterization!$J$17 + G123*characterization!$J$15</f>
+        <f>F123*characterization!$L$17 + G123*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L123" s="7">
@@ -11390,7 +11888,7 @@
         </is>
       </c>
       <c r="I124" s="7">
-        <f>F124*characterization!$D$17 + G124*characterization!$D$15</f>
+        <f>F124*characterization!$B$17 + G124*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J124" s="7">
@@ -11398,7 +11896,7 @@
         <v/>
       </c>
       <c r="K124" s="7">
-        <f>F124*characterization!$J$17 + G124*characterization!$J$15</f>
+        <f>F124*characterization!$L$17 + G124*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L124" s="7">
@@ -11465,7 +11963,7 @@
         </is>
       </c>
       <c r="I125" s="7">
-        <f>F125*characterization!$D$17 + G125*characterization!$D$15</f>
+        <f>F125*characterization!$B$17 + G125*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J125" s="7">
@@ -11473,7 +11971,7 @@
         <v/>
       </c>
       <c r="K125" s="7">
-        <f>F125*characterization!$J$17 + G125*characterization!$J$15</f>
+        <f>F125*characterization!$L$17 + G125*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L125" s="7">
@@ -11540,7 +12038,7 @@
         </is>
       </c>
       <c r="I126" s="7">
-        <f>F126*characterization!$D$17 + G126*characterization!$D$15</f>
+        <f>F126*characterization!$B$17 + G126*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J126" s="7">
@@ -11548,7 +12046,7 @@
         <v/>
       </c>
       <c r="K126" s="7">
-        <f>F126*characterization!$J$17 + G126*characterization!$J$15</f>
+        <f>F126*characterization!$L$17 + G126*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L126" s="7">
@@ -11615,7 +12113,7 @@
         </is>
       </c>
       <c r="I127" s="7">
-        <f>F127*characterization!$D$17 + G127*characterization!$D$15</f>
+        <f>F127*characterization!$B$17 + G127*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J127" s="7">
@@ -11623,7 +12121,7 @@
         <v/>
       </c>
       <c r="K127" s="7">
-        <f>F127*characterization!$J$17 + G127*characterization!$J$15</f>
+        <f>F127*characterization!$L$17 + G127*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L127" s="7">
@@ -11690,7 +12188,7 @@
         </is>
       </c>
       <c r="I128" s="7">
-        <f>F128*characterization!$D$17 + G128*characterization!$D$15</f>
+        <f>F128*characterization!$B$17 + G128*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J128" s="7">
@@ -11698,7 +12196,7 @@
         <v/>
       </c>
       <c r="K128" s="7">
-        <f>F128*characterization!$J$17 + G128*characterization!$J$15</f>
+        <f>F128*characterization!$L$17 + G128*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L128" s="7">
@@ -11765,7 +12263,7 @@
         </is>
       </c>
       <c r="I129" s="7">
-        <f>F129*characterization!$D$17 + G129*characterization!$D$15</f>
+        <f>F129*characterization!$B$17 + G129*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J129" s="7">
@@ -11773,7 +12271,7 @@
         <v/>
       </c>
       <c r="K129" s="7">
-        <f>F129*characterization!$J$17 + G129*characterization!$J$15</f>
+        <f>F129*characterization!$L$17 + G129*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L129" s="7">
@@ -11840,7 +12338,7 @@
         </is>
       </c>
       <c r="I130" s="7">
-        <f>F130*characterization!$D$17 + G130*characterization!$D$15</f>
+        <f>F130*characterization!$B$17 + G130*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J130" s="7">
@@ -11848,7 +12346,7 @@
         <v/>
       </c>
       <c r="K130" s="7">
-        <f>F130*characterization!$J$17 + G130*characterization!$J$15</f>
+        <f>F130*characterization!$L$17 + G130*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L130" s="7">
@@ -11915,7 +12413,7 @@
         </is>
       </c>
       <c r="I131" s="7">
-        <f>F131*characterization!$D$17 + G131*characterization!$D$15</f>
+        <f>F131*characterization!$B$17 + G131*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J131" s="7">
@@ -11923,7 +12421,7 @@
         <v/>
       </c>
       <c r="K131" s="7">
-        <f>F131*characterization!$J$17 + G131*characterization!$J$15</f>
+        <f>F131*characterization!$L$17 + G131*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L131" s="7">
@@ -11990,7 +12488,7 @@
         </is>
       </c>
       <c r="I132" s="7">
-        <f>F132*characterization!$D$17 + G132*characterization!$D$15</f>
+        <f>F132*characterization!$B$17 + G132*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J132" s="7">
@@ -11998,7 +12496,7 @@
         <v/>
       </c>
       <c r="K132" s="7">
-        <f>F132*characterization!$J$17 + G132*characterization!$J$15</f>
+        <f>F132*characterization!$L$17 + G132*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L132" s="7">
@@ -12069,7 +12567,7 @@
         </is>
       </c>
       <c r="I133" s="7">
-        <f>F133*characterization!$D$17 + G133*characterization!$D$15</f>
+        <f>F133*characterization!$B$17 + G133*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J133" s="7">
@@ -12077,7 +12575,7 @@
         <v/>
       </c>
       <c r="K133" s="7">
-        <f>F133*characterization!$J$17 + G133*characterization!$J$15</f>
+        <f>F133*characterization!$L$17 + G133*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L133" s="7">
@@ -12148,7 +12646,7 @@
         </is>
       </c>
       <c r="I134" s="7">
-        <f>F134*characterization!$D$17 + G134*characterization!$D$15</f>
+        <f>F134*characterization!$B$17 + G134*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J134" s="7">
@@ -12156,7 +12654,7 @@
         <v/>
       </c>
       <c r="K134" s="7">
-        <f>F134*characterization!$J$17 + G134*characterization!$J$15</f>
+        <f>F134*characterization!$L$17 + G134*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L134" s="7">
@@ -12227,7 +12725,7 @@
         </is>
       </c>
       <c r="I135" s="7">
-        <f>F135*characterization!$D$17 + G135*characterization!$D$15</f>
+        <f>F135*characterization!$B$17 + G135*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J135" s="7">
@@ -12235,7 +12733,7 @@
         <v/>
       </c>
       <c r="K135" s="7">
-        <f>F135*characterization!$J$17 + G135*characterization!$J$15</f>
+        <f>F135*characterization!$L$17 + G135*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L135" s="7">
@@ -12306,7 +12804,7 @@
         </is>
       </c>
       <c r="I136" s="7">
-        <f>F136*characterization!$D$17 + G136*characterization!$D$15</f>
+        <f>F136*characterization!$B$17 + G136*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J136" s="7">
@@ -12314,7 +12812,7 @@
         <v/>
       </c>
       <c r="K136" s="7">
-        <f>F136*characterization!$J$17 + G136*characterization!$J$15</f>
+        <f>F136*characterization!$L$17 + G136*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L136" s="7">
@@ -12385,7 +12883,7 @@
         </is>
       </c>
       <c r="I137" s="7">
-        <f>F137*characterization!$D$17 + G137*characterization!$D$15</f>
+        <f>F137*characterization!$B$17 + G137*characterization!$B$15</f>
         <v/>
       </c>
       <c r="J137" s="7">
@@ -12393,7 +12891,7 @@
         <v/>
       </c>
       <c r="K137" s="7">
-        <f>F137*characterization!$J$17 + G137*characterization!$J$15</f>
+        <f>F137*characterization!$L$17 + G137*characterization!$L$15</f>
         <v/>
       </c>
       <c r="L137" s="7">

</xml_diff>

<commit_message>
feat(timing_char/work): bump sweep grid to 2.0-3.0 GHz
User reports the 1-2 GHz range still keeps everything passing.  Shifting
the grid up to where ASAP7 RVT will actually start to choke on real chains:

  columns: TT_2000 / TT_2250 / TT_2500 / TT_2750 / TT_3000
           FF_2000 / FF_2250 / FF_2500 / FF_2750 / FF_3000
           SS_2000 / SS_2250 / SS_2500 / SS_2750 / SS_3000

Sample TT-corner Max-levels-per-cycle ranges over the new grid:
  NAND:  66 -> 43
  MUX:   29 -> 19   (one MUX2 ~ 16.3 ps; only 19 levels fit at 333 ps)
  XOR:   18 -> 12
  MULT:  16 -> 10   (the mixed-bag proxy hits 10 levels at 3 GHz TT)
  CARRY: 15 -> 10

At 3 GHz SS corner the budget gets very tight:
  NAND: 27 / MUX: 12 / XOR: 7 / MULT: 8 / CARRY: 7

This is where designs start failing without aggressive pipelining and
critical-path muxing rework.
</commit_message>
<xml_diff>
--- a/projects/components/timing_characterization/work/asap7_characterization.xlsx
+++ b/projects/components/timing_characterization/work/asap7_characterization.xlsx
@@ -512,77 +512,77 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>TT_1000MHz</t>
+          <t>TT_2000MHz</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>TT_1250MHz</t>
+          <t>TT_2250MHz</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>TT_1500MHz</t>
+          <t>TT_2500MHz</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>TT_1750MHz</t>
+          <t>TT_2750MHz</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>TT_2000MHz</t>
+          <t>TT_3000MHz</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>FF_1000MHz</t>
+          <t>FF_2000MHz</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>FF_1250MHz</t>
+          <t>FF_2250MHz</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>FF_1500MHz</t>
+          <t>FF_2500MHz</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>FF_1750MHz</t>
+          <t>FF_2750MHz</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>FF_2000MHz</t>
+          <t>FF_3000MHz</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>SS_1000MHz</t>
+          <t>SS_2000MHz</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>SS_1250MHz</t>
+          <t>SS_2250MHz</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>SS_1500MHz</t>
+          <t>SS_2500MHz</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>SS_1750MHz</t>
+          <t>SS_2750MHz</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>SS_2000MHz</t>
+          <t>SS_3000MHz</t>
         </is>
       </c>
     </row>
@@ -593,49 +593,49 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>800</v>
+        <v>444.4</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>666.7</v>
+        <v>400</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>571.4</v>
+        <v>363.6</v>
       </c>
       <c r="F2" s="2" t="n">
+        <v>333.3</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>1000</v>
-      </c>
       <c r="H2" s="2" t="n">
-        <v>800</v>
+        <v>444.4</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>666.7</v>
+        <v>400</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>571.4</v>
+        <v>363.6</v>
       </c>
       <c r="K2" s="2" t="n">
+        <v>333.3</v>
+      </c>
+      <c r="L2" s="2" t="n">
         <v>500</v>
       </c>
-      <c r="L2" s="2" t="n">
-        <v>1000</v>
-      </c>
       <c r="M2" s="2" t="n">
-        <v>800</v>
+        <v>444.4</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>666.7</v>
+        <v>400</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>571.4</v>
+        <v>363.6</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>500</v>
+        <v>333.3</v>
       </c>
     </row>
     <row r="3">
@@ -737,49 +737,49 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>135</v>
+        <v>66</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>107</v>
+        <v>58</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>89</v>
+        <v>52</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>76</v>
+        <v>47</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>166</v>
+        <v>82</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>133</v>
+        <v>73</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>110</v>
+        <v>65</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>94</v>
+        <v>59</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>82</v>
+        <v>54</v>
       </c>
       <c r="L6" s="2" t="n">
-        <v>85</v>
+        <v>41</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>41</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
@@ -789,49 +789,49 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="D7" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="I7" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="J7" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="K7" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="F7" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="I7" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="J7" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>30</v>
-      </c>
       <c r="L7" s="2" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="M7" s="2" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="P7" s="2" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -841,49 +841,49 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="D8" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H8" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="E8" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="F8" s="2" t="n">
+      <c r="I8" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="K8" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="G8" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="J8" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>44</v>
-      </c>
       <c r="L8" s="2" t="n">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="M8" s="2" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="P8" s="2" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -893,49 +893,49 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E9" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I9" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="J9" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="K9" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="I9" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="J9" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="K9" s="2" t="n">
-        <v>23</v>
-      </c>
       <c r="L9" s="2" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="P9" s="2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -945,49 +945,49 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F10" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="I10" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="J10" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="G10" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="H10" s="5" t="n">
-        <v>36</v>
-      </c>
-      <c r="I10" s="5" t="n">
-        <v>30</v>
-      </c>
-      <c r="J10" s="5" t="n">
-        <v>25</v>
-      </c>
       <c r="K10" s="5" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -997,49 +997,49 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -1049,49 +1049,49 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>84</v>
+        <v>41</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>67</v>
+        <v>36</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="P12" s="2" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
feat(timing_char/work): bold red font on negative slack cells
Added conditional formatting to both downstream sheets so failing paths
jump out at a glance:

  building blocks  slack column AF3:AF11    bold + #C00000 if slack < 0
  stream           slack column R3:R137     bold + #C00000 if slack < 0

When you walk the Design clocks freq up the sweep range, any row whose
slack flips negative will now show in bold dark red.  Easy visual scan
for which FUB ports break first at the planned freq.
</commit_message>
<xml_diff>
--- a/projects/components/timing_characterization/work/asap7_characterization.xlsx
+++ b/projects/components/timing_characterization/work/asap7_characterization.xlsx
@@ -122,6 +122,14 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00C00000"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -3317,6 +3325,11 @@
     <mergeCell ref="B2:AG2"/>
     <mergeCell ref="A3:AG3"/>
   </mergeCells>
+  <conditionalFormatting sqref="AF3:AF11">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12999,6 +13012,11 @@
     <mergeCell ref="A140:S140"/>
     <mergeCell ref="A64:S64"/>
   </mergeCells>
+  <conditionalFormatting sqref="R3:R137">
+    <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>